<commit_message>
Fill the phone number to excel
</commit_message>
<xml_diff>
--- a/Pruebas_Homologacion_PS_3G_4G.xlsx
+++ b/Pruebas_Homologacion_PS_3G_4G.xlsx
@@ -2127,7 +2127,7 @@
       <c r="D14" s="134" t="n"/>
       <c r="F14" s="74" t="inlineStr">
         <is>
-          <t>Línea Pospago: 5530760949</t>
+          <t>Línea Pospago: 5523427847</t>
         </is>
       </c>
       <c r="G14" s="133" t="n"/>
@@ -2136,7 +2136,7 @@
     <row r="15" ht="15.5" customHeight="1" thickBot="1" thickTop="1">
       <c r="B15" s="132" t="inlineStr">
         <is>
-          <t>Modelo: V2543</t>
+          <t>Modelo: V2515</t>
         </is>
       </c>
       <c r="C15" s="133" t="n"/>
@@ -2152,7 +2152,7 @@
     <row r="16" ht="15.5" customHeight="1" thickBot="1" thickTop="1">
       <c r="B16" s="132" t="inlineStr">
         <is>
-          <t>Fecha de pruebas: 02/03/2026</t>
+          <t>Fecha de pruebas: 25/05/2026</t>
         </is>
       </c>
       <c r="C16" s="133" t="n"/>
@@ -2238,11 +2238,15 @@
           <t>MMS</t>
         </is>
       </c>
-      <c r="C21" s="42" t="n">
-        <v>0.5638888888888889</v>
-      </c>
-      <c r="D21" s="41" t="n">
-        <v>0.5770833333333333</v>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>01:18 PM</t>
+        </is>
+      </c>
+      <c r="D21" s="41" t="inlineStr">
+        <is>
+          <t>01:19 PM</t>
+        </is>
       </c>
       <c r="E21" s="42" t="n">
         <v>0.59375</v>
@@ -2535,12 +2539,12 @@
       </c>
       <c r="C36" s="51" t="inlineStr">
         <is>
-          <t>11:50 AM</t>
+          <t>01:18 PM</t>
         </is>
       </c>
       <c r="D36" s="51" t="inlineStr">
         <is>
-          <t>11:51 AM</t>
+          <t>01:19 PM</t>
         </is>
       </c>
       <c r="E36" s="31" t="n"/>

</xml_diff>

<commit_message>
Twitter 3G SS Fix
</commit_message>
<xml_diff>
--- a/Pruebas_Homologacion_PS_3G_4G.xlsx
+++ b/Pruebas_Homologacion_PS_3G_4G.xlsx
@@ -2333,11 +2333,15 @@
       <c r="F24" s="47" t="n">
         <v>0.6486111111111111</v>
       </c>
-      <c r="G24" s="62" t="n">
-        <v>0.8104166666666667</v>
-      </c>
-      <c r="H24" s="62" t="n">
-        <v>0.8131944444444444</v>
+      <c r="G24" s="62" t="inlineStr">
+        <is>
+          <t>03:19 PM</t>
+        </is>
+      </c>
+      <c r="H24" s="62" t="inlineStr">
+        <is>
+          <t>03:23 PM</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="15.5" customHeight="1" thickBot="1" thickTop="1">
@@ -4082,8 +4086,10 @@
       <c r="S96" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="T96" s="41" t="n">
-        <v>0.8104166666666667</v>
+      <c r="T96" s="41" t="inlineStr">
+        <is>
+          <t>03:19 PM</t>
+        </is>
       </c>
       <c r="V96" s="148" t="n"/>
       <c r="X96" s="149" t="n"/>
@@ -4092,8 +4098,10 @@
       <c r="S97" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="T97" s="62" t="n">
-        <v>0.8111111111111111</v>
+      <c r="T97" s="62" t="inlineStr">
+        <is>
+          <t>03:20 PM</t>
+        </is>
       </c>
       <c r="V97" s="148" t="n"/>
       <c r="X97" s="149" t="n"/>
@@ -4102,8 +4110,10 @@
       <c r="S98" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="T98" s="41" t="n">
-        <v>0.8118055555555556</v>
+      <c r="T98" s="41" t="inlineStr">
+        <is>
+          <t>03:21 PM</t>
+        </is>
       </c>
       <c r="V98" s="148" t="n"/>
       <c r="X98" s="149" t="n"/>
@@ -4112,8 +4122,10 @@
       <c r="S99" s="54" t="n">
         <v>4</v>
       </c>
-      <c r="T99" s="62" t="n">
-        <v>0.8125</v>
+      <c r="T99" s="62" t="inlineStr">
+        <is>
+          <t>03:22 PM</t>
+        </is>
       </c>
       <c r="V99" s="148" t="n"/>
       <c r="X99" s="149" t="n"/>
@@ -4122,8 +4134,10 @@
       <c r="S100" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="T100" s="41" t="n">
-        <v>0.8131944444444444</v>
+      <c r="T100" s="41" t="inlineStr">
+        <is>
+          <t>03:23 PM</t>
+        </is>
       </c>
       <c r="U100" s="31" t="n"/>
       <c r="V100" s="148" t="n"/>

</xml_diff>